<commit_message>
apache poi output excel based on annotation for admin manuals template
</commit_message>
<xml_diff>
--- a/output.xlsx
+++ b/output.xlsx
@@ -14,7 +14,7 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="18">
   <si>
-    <t>Group 1</t>
+    <t>1</t>
   </si>
   <si>
     <t>Group 1 Optional Name</t>
@@ -32,7 +32,7 @@
     <t>Attribute 2 Value</t>
   </si>
   <si>
-    <t>Group 2</t>
+    <t>2</t>
   </si>
   <si>
     <t>String List</t>

</xml_diff>